<commit_message>
Restore TCM/Care Gaps/COPD/CHF and make Beyond Health conversational.
Bring back Care Gaps, COPD, and CHF as dropdown programs alongside TCM, retire
the Cedars numeric inpatient template, and rewrite Beyond Health SMS copy to
natural-language conversational AI replies with no numbered menus or em dashes.

Co-authored-by: kiannuzzi-byte <kiannuzzi-byte@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/BH-GLP1-Program-Continuity-SMS.xlsx
+++ b/BH-GLP1-Program-Continuity-SMS.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -452,14 +452,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Hi {patient}, this is {hospital}. We're checking in on your weight management / GLP-1 program.
-Reply 1 to continue in English.
-Reply STOP to opt out.</t>
+          <t>Hi {patient}, this is {hospital}. We're checking in on your weight management program and have a few quick questions about how things are going.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1 — Continue</t>
+          <t>hey yes this is Maria</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -471,148 +469,188 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Thanks. This is a quick check-in from your Beyond Health care team — it only takes about a minute.
-Are we reaching {patient}?
-Reply 1 if this is the patient.
-Reply 2 if you are a caregiver.
-Reply 3 if wrong number.</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1 — Yes, this is Maria</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2.0</t>
-        </is>
-      </c>
+          <t>Before we continue, are we texting with {patient}, a caregiver, or did we reach the wrong number?</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Great, thanks {patient}.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>yeah I've been taking it like they told me</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>2.0</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Great, thank you {patient}.
-Our records show you are enrolled in Beyond Health's weight management program and are due for your Week-4 check-in with your care team.
-Have you been able to take your prescribed medication as directed?
-Reply 1 if yes — taking it as directed.
-Reply 2 if you have missed doses or stopped.
-Reply 3 if you have not been able to obtain your medication.</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1 — Yes, I am taking it</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>3.0</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Thanks for confirming.
-Are you having any side effects that concern you (for example nausea, vomiting, dizziness, or stomach pain)?
-Reply 1 if you are doing fine — no concerning side effects.
-Reply 2 if you are having side effects or have questions for the care team.</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>2 — Yes, I have been nauseous and it is getting worse</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>4.0</t>
-        </is>
-      </c>
+          <t>Our records show you're enrolled in Beyond Health's weight management program and you're due for your Week 4 check-in. Have you been able to take your prescribed medication as directed?</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>We're sorry you're dealing with that — thank you for letting us know. A member of your Beyond Health care team will follow up.
-If this feels urgent, please call the clinic at (505) 899-4414 or seek emergency care.
-You also have coach and nutrition visits as part of your program. Were you able to keep your most recent coach or nutrition appointment?
-Reply 1 if yes — completed.
-Reply 2 if you missed it or need to reschedule.
-Reply 3 if you are not sure / need help.</t>
+          <t>Thanks for letting us know.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2 — I missed my nutrition visit last week</t>
+          <t>honestly the nausea has been pretty bad and it's getting worse</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>3.0</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Got it — we want to get you back on track. Would you like someone from Beyond Health to call you back to discuss side effects and help reschedule your coach or nutrition visit?
-Reply 1 if yes, please call me back.
-Reply 2 if no, I'm all set for now.</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>1 — Yes, please call me back</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>6.0</t>
-        </is>
-      </c>
+          <t>Are you having any side effects that concern you, like nausea, vomiting, dizziness, or stomach pain?</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Thank you. We've flagged your responses for the care team and someone will reach out soon during clinic hours.
-Quick tip: small, frequent meals and staying hydrated can help with nausea — your coach can tailor this with you.
-Reply HELP for help. Reply STOP to unsubscribe.
-Thank you for partnering with Beyond Health on your health goals.</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
+          <t>I'm sorry you're dealing with that, thank you for telling us. Someone from your Beyond Health care team will follow up. If this feels urgent, please call the clinic at (505) 899-4414 or seek emergency care.</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>no I missed the nutrition one last week, things got crazy</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>You also have coach and nutrition visits as part of your program. Were you able to keep your most recent coach or nutrition appointment?</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Got it, we want to help get you back on track. Would you like someone from Beyond Health to call you back to talk through the side effects and help reschedule your coach or nutrition visit?</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>yes please call me when you can</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Thank you. We've flagged this for the care team and someone will reach out during clinic hours.</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Quick tip while you wait: smaller meals more often and staying hydrated can help with nausea. Your coach can tailor that with you.</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Reply HELP for help. Reply STOP to unsubscribe. Thanks for partnering with Beyond Health on your health goals.</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>